<commit_message>
Update reference files and data outputs for inventory integration
- Updated General_Journal.xlsx and General_Ledger_edited.xlsx reference files
- Updated adjusting_entries_Jan2026.xlsx with inventory reference sheet
- Updated ledger_summary_Jan2026.xlsx with inventory summary

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/accountant-skill/data/Jan2026/adjusting_entries_Jan2026.xlsx
+++ b/accountant-skill/data/Jan2026/adjusting_entries_Jan2026.xlsx
@@ -12,8 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank Recon Entries" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accruals" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prepayments" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Entries" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account Impact" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Entries" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account Impact" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -132,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -162,6 +163,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -2094,6 +2096,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Inventory — Materials Issued to Production</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Summary of inventory sub-ledger movements</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-01  to  2026-01-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Materials issued to production are recorded via inventory sub-ledgers. Cost of materials used flows to COGS accounts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>No inventory sub-ledger data found for this period.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="004472C4"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2503,7 +2561,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0070AD47"/>
@@ -2611,13 +2669,13 @@
       <c r="E6" s="7" t="n">
         <v>1438500</v>
       </c>
-      <c r="F6" s="13" t="n">
+      <c r="F6" s="14" t="n">
         <v>-3000</v>
       </c>
       <c r="G6" s="7" t="n">
         <v>1435500</v>
       </c>
-      <c r="H6" s="14" t="n">
+      <c r="H6" s="15" t="n">
         <v>-0.002085505735140772</v>
       </c>
     </row>
@@ -2651,7 +2709,7 @@
       <c r="G7" s="7" t="n">
         <v>518750</v>
       </c>
-      <c r="H7" s="14" t="n">
+      <c r="H7" s="15" t="n">
         <v>0.0375</v>
       </c>
     </row>
@@ -2685,7 +2743,7 @@
       <c r="G8" s="7" t="n">
         <v>472500</v>
       </c>
-      <c r="H8" s="14" t="n">
+      <c r="H8" s="15" t="n">
         <v>0.05</v>
       </c>
     </row>
@@ -2719,7 +2777,7 @@
       <c r="G9" s="7" t="n">
         <v>113500</v>
       </c>
-      <c r="H9" s="14" t="n">
+      <c r="H9" s="15" t="n">
         <v>0.135</v>
       </c>
     </row>
@@ -2753,7 +2811,7 @@
       <c r="G10" s="7" t="n">
         <v>1486500</v>
       </c>
-      <c r="H10" s="14" t="n">
+      <c r="H10" s="15" t="n">
         <v>0.01225740551583248</v>
       </c>
     </row>
@@ -2787,7 +2845,7 @@
       <c r="G11" s="7" t="n">
         <v>54750</v>
       </c>
-      <c r="H11" s="15" t="inlineStr">
+      <c r="H11" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -2823,7 +2881,7 @@
       <c r="G12" s="7" t="n">
         <v>15000</v>
       </c>
-      <c r="H12" s="15" t="inlineStr">
+      <c r="H12" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>